<commit_message>
Collect initial data: - Actualicé scrapers de sofifa y whoscored (aun queda revisar si estan bien los datos) - Meti los scrapers en la carpeta collect_initial_data. - En main.py planeo quitar la extraccion de Flashscore y agregar la de sofifa.
</commit_message>
<xml_diff>
--- a/p2_data_understanding/data/df_competencias.xlsx
+++ b/p2_data_understanding/data/df_competencias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C26F3005-0924-3B4C-B3BA-9FE750FE1531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84946963-31C3-4642-B78C-F7B64A26D501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15740" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,88 +36,40 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>pais</t>
   </si>
   <si>
-    <t>Argentina</t>
-  </si>
-  <si>
     <t>cod_pais</t>
   </si>
   <si>
-    <t>Liga Profesional</t>
-  </si>
-  <si>
     <t>competicion</t>
   </si>
   <si>
     <t>cod_competicion</t>
   </si>
   <si>
-    <t>Copa de la Superliga</t>
-  </si>
-  <si>
-    <t>Italy</t>
-  </si>
-  <si>
-    <t>Serie A</t>
-  </si>
-  <si>
     <t>England</t>
   </si>
   <si>
+    <t>is_cup</t>
+  </si>
+  <si>
+    <t>Community Shield</t>
+  </si>
+  <si>
+    <t>FA Cup</t>
+  </si>
+  <si>
     <t>Premier League</t>
-  </si>
-  <si>
-    <t>Super Cup</t>
-  </si>
-  <si>
-    <t>Cup</t>
-  </si>
-  <si>
-    <t>South America</t>
-  </si>
-  <si>
-    <t>Copa Sudamericana</t>
-  </si>
-  <si>
-    <t>Recopa Sudamericana</t>
-  </si>
-  <si>
-    <t>Copa Libertadores</t>
-  </si>
-  <si>
-    <t>competicion_fs</t>
-  </si>
-  <si>
-    <t>is_cup</t>
-  </si>
-  <si>
-    <t>Copa Argentina</t>
-  </si>
-  <si>
-    <t>Supercopa</t>
-  </si>
-  <si>
-    <t>pais_fs</t>
-  </si>
-  <si>
-    <t>Sudamerica</t>
-  </si>
-  <si>
-    <t>Inglaterra</t>
-  </si>
-  <si>
-    <t>Italia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -129,6 +81,14 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -151,14 +111,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -471,242 +434,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3570E4A9-1B7C-CD4C-90F1-ACEB6414EE21}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="23.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>252</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
       <c r="C2">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" t="s">
-        <v>3</v>
-      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>11</v>
+        <v>252</v>
       </c>
       <c r="B3" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>504</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="F3" t="s">
-        <v>1</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>11</v>
+        <v>252</v>
       </c>
       <c r="B4" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C4">
-        <v>541</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
-      <c r="F4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
-      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>11</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>697</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5" t="s">
-        <v>1</v>
-      </c>
-      <c r="G5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>108</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6">
-        <v>5</v>
-      </c>
-      <c r="D6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>252</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-      <c r="D7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="s">
-        <v>23</v>
-      </c>
-      <c r="G7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>265</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8">
-        <v>105</v>
-      </c>
-      <c r="D8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>265</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9">
-        <v>146</v>
-      </c>
-      <c r="D9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>265</v>
-      </c>
-      <c r="B10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10">
-        <v>271</v>
-      </c>
-      <c r="D10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" t="s">
-        <v>15</v>
-      </c>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C8" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Collect initial data: - Datos solo de Flashscore y Sofifa (ya no de WhoScored) - Ya no extraigo todos los datos de Flashscore juntos sino que separo en df_part y df_part_jug para mejorar el manejo de los datos.
</commit_message>
<xml_diff>
--- a/p2_data_understanding/data/df_competencias.xlsx
+++ b/p2_data_understanding/data/df_competencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84946963-31C3-4642-B78C-F7B64A26D501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF2C6773-AAEB-A64B-AAD7-E184854EC22E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -56,13 +56,13 @@
     <t>is_cup</t>
   </si>
   <si>
-    <t>Community Shield</t>
-  </si>
-  <si>
     <t>FA Cup</t>
   </si>
   <si>
     <t>Premier League</t>
+  </si>
+  <si>
+    <t>FA Community Shield</t>
   </si>
 </sst>
 </file>
@@ -469,7 +469,7 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -486,7 +486,7 @@
         <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -503,7 +503,7 @@
         <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4">
         <v>1</v>

</xml_diff>

<commit_message>
Corrida de todo el main.py usando datos de la Premier desde 2014/15 al 2024 para tener idea de precision inicial. Precision test de 54.4%. Muy alentador.
</commit_message>
<xml_diff>
--- a/p2_data_understanding/data/df_competencias.xlsx
+++ b/p2_data_understanding/data/df_competencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF2C6773-AAEB-A64B-AAD7-E184854EC22E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30827818-DB69-864B-A054-93269FAA76DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="18660" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -59,10 +59,10 @@
     <t>FA Cup</t>
   </si>
   <si>
-    <t>Premier League</t>
-  </si>
-  <si>
     <t>FA Community Shield</t>
+  </si>
+  <si>
+    <t>championship</t>
   </si>
 </sst>
 </file>
@@ -434,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3570E4A9-1B7C-CD4C-90F1-ACEB6414EE21}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="23.5" bestFit="1" customWidth="1"/>
@@ -466,13 +466,13 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -483,10 +483,10 @@
         <v>4</v>
       </c>
       <c r="C3">
-        <v>96</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -499,18 +499,15 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4">
-        <v>26</v>
-      </c>
       <c r="D4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C8" s="2"/>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Me quedo con los datasets de seguridad que necesito
</commit_message>
<xml_diff>
--- a/p2_data_understanding/data/df_competencias.xlsx
+++ b/p2_data_understanding/data/df_competencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30827818-DB69-864B-A054-93269FAA76DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E28EB5-4542-6B48-BD94-8A22F93C1A39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="18660" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t>pais</t>
   </si>
@@ -59,10 +59,16 @@
     <t>FA Cup</t>
   </si>
   <si>
+    <t>Premier League</t>
+  </si>
+  <si>
     <t>FA Community Shield</t>
   </si>
   <si>
-    <t>championship</t>
+    <t>EFL Cup</t>
+  </si>
+  <si>
+    <t>Championship</t>
   </si>
 </sst>
 </file>
@@ -434,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3570E4A9-1B7C-CD4C-90F1-ACEB6414EE21}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="23.5" bestFit="1" customWidth="1"/>
@@ -466,13 +472,13 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>96</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -483,10 +489,10 @@
         <v>4</v>
       </c>
       <c r="C3">
-        <v>26</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -499,15 +505,46 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
+      <c r="C4">
+        <v>26</v>
+      </c>
       <c r="D4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>252</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>252</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C7" s="2"/>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C8" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Agrego competeencias de Argentina y quito las columnas de codigo de pais y de competicion (creo que eran para Whoscored)
</commit_message>
<xml_diff>
--- a/p2_data_understanding/data/df_competencias.xlsx
+++ b/p2_data_understanding/data/df_competencias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E28EB5-4542-6B48-BD94-8A22F93C1A39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E2F46B-F3A0-384D-ABB3-BD55665F4658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="18660" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,20 +36,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
   <si>
     <t>pais</t>
   </si>
   <si>
-    <t>cod_pais</t>
-  </si>
-  <si>
     <t>competicion</t>
   </si>
   <si>
-    <t>cod_competicion</t>
-  </si>
-  <si>
     <t>England</t>
   </si>
   <si>
@@ -69,13 +63,37 @@
   </si>
   <si>
     <t>Championship</t>
+  </si>
+  <si>
+    <t>Argentina</t>
+  </si>
+  <si>
+    <t>Liga Profesional</t>
+  </si>
+  <si>
+    <t>Copa de la Liga Profesional</t>
+  </si>
+  <si>
+    <t>Primera Nacional</t>
+  </si>
+  <si>
+    <t>Copa Argentina</t>
+  </si>
+  <si>
+    <t>Supercopa</t>
+  </si>
+  <si>
+    <t>Supercopa Internacional</t>
+  </si>
+  <si>
+    <t>Trofeo de Campeones</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -87,14 +105,6 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -117,17 +127,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -440,111 +447,155 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3570E4A9-1B7C-CD4C-90F1-ACEB6414EE21}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>252</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
       <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>252</v>
-      </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C3">
-        <v>96</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>252</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4">
-        <v>26</v>
-      </c>
-      <c r="D4" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>252</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>252</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="B7" t="s">
         <v>10</v>
       </c>
-      <c r="E6">
+      <c r="C7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C8" s="2"/>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Cambios en ultimos dias
</commit_message>
<xml_diff>
--- a/p2_data_understanding/data/df_competencias.xlsx
+++ b/p2_data_understanding/data/df_competencias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E2F46B-F3A0-384D-ABB3-BD55665F4658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{168B6760-3991-6447-A62F-5002FF7E0120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15700" xr2:uid="{7E04431C-C58B-6A45-9218-66EB9A490B36}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,13 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
-  <si>
-    <t>pais</t>
-  </si>
-  <si>
-    <t>competicion</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="30">
   <si>
     <t>England</t>
   </si>
@@ -87,6 +81,51 @@
   </si>
   <si>
     <t>Trofeo de Campeones</t>
+  </si>
+  <si>
+    <t>Serie A</t>
+  </si>
+  <si>
+    <t>Copa Italia</t>
+  </si>
+  <si>
+    <t>competicion_sofifa</t>
+  </si>
+  <si>
+    <t>espana</t>
+  </si>
+  <si>
+    <t>La Liga</t>
+  </si>
+  <si>
+    <t>LaLiga EA Sports</t>
+  </si>
+  <si>
+    <t>Copa del Rey</t>
+  </si>
+  <si>
+    <t>Liga Profesional de Fútbol</t>
+  </si>
+  <si>
+    <t>competicion_flashscore</t>
+  </si>
+  <si>
+    <t>pais_sofifa</t>
+  </si>
+  <si>
+    <t>Inglaterra</t>
+  </si>
+  <si>
+    <t>pais_flashscore</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>Italia</t>
+  </si>
+  <si>
+    <t>Spain</t>
   </si>
 </sst>
 </file>
@@ -130,9 +169,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,154 +489,297 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3570E4A9-1B7C-CD4C-90F1-ACEB6414EE21}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
         <v>13</v>
       </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" t="s">
         <v>14</v>
       </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" t="s">
         <v>15</v>
       </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
         <v>16</v>
       </c>
-      <c r="C13">
-        <v>1</v>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>